<commit_message>
feat: Adaptive Momentum Regression & continuous multi-year 2030 projections (unified_plan_metrics_template.xlsx)
</commit_message>
<xml_diff>
--- a/unified_plan_metrics_template.xlsx
+++ b/unified_plan_metrics_template.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://chaffeyccd-my.sharepoint.com/personal/joseph_cascio_chaffey_edu/Documents/Research Analyst/Surveys and Reports/Combining Initiative Reports/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://chaffeyccd-my.sharepoint.com/personal/joseph_cascio_chaffey_edu/Documents/Desktop/Dashboards/Plan Metrics Dashboard/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="435" documentId="8_{0966D836-5100-49BC-8A45-6686B0C0AF40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F6475197-4B75-4748-AD3B-1CB5A3E6C027}"/>
+  <xr:revisionPtr revIDLastSave="436" documentId="8_{0966D836-5100-49BC-8A45-6686B0C0AF40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{13D647DB-FF79-4BD1-9D4F-8D1789A2B7AE}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{BFF79AE2-E76B-441F-B8D7-30B63CE1804C}"/>
   </bookViews>
@@ -1047,9 +1047,6 @@
     <t>Strategic Plan Target Goal (By 2030)</t>
   </si>
   <si>
-    <t>EMP Target Goal (By YYYY)</t>
-  </si>
-  <si>
     <t>IR Dashboard - Enrollment Management</t>
   </si>
   <si>
@@ -1111,6 +1108,9 @@
   </si>
   <si>
     <t>CCFS-320 Report</t>
+  </si>
+  <si>
+    <t>EMP Target Goal (By 2030)</t>
   </si>
 </sst>
 </file>
@@ -1740,7 +1740,7 @@
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -1911,15 +1911,6 @@
     <xf numFmtId="0" fontId="16" fillId="37" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="44">
     <cellStyle name="20% - Accent1" xfId="20" builtinId="30" customBuiltin="1"/>
@@ -2729,7 +2720,7 @@
     <tableColumn id="9" xr3:uid="{F5EAFEFD-FC0A-487F-8525-1C93255BD17F}" name="2025-2026" dataDxfId="24"/>
     <tableColumn id="28" xr3:uid="{71F30DCF-07A1-4BBA-8536-EA45043CB21E}" name="Date Pulled" dataDxfId="23" dataCellStyle="Percent"/>
     <tableColumn id="22" xr3:uid="{19854763-5938-48CE-8523-23258BFF1C3E}" name="EMP Baseline (2025-2026 Yr 0)" dataDxfId="22"/>
-    <tableColumn id="23" xr3:uid="{14F0D8E9-D836-4B80-94D3-7B8418392D1A}" name="EMP Target Goal (By YYYY)" dataDxfId="21"/>
+    <tableColumn id="23" xr3:uid="{14F0D8E9-D836-4B80-94D3-7B8418392D1A}" name="EMP Target Goal (By 2030)" dataDxfId="21"/>
     <tableColumn id="24" xr3:uid="{FA021FCD-2B93-4B93-B866-74FFE5B66D07}" name="Strategic Plan Baseline (2024-2025 Yr 0)" dataDxfId="20"/>
     <tableColumn id="25" xr3:uid="{D5AB3269-32D4-42B9-BB3A-AA4B7E4FFDFF}" name="Strategic Plan Target Goal (By 2030)" dataDxfId="19"/>
     <tableColumn id="10" xr3:uid="{75661E75-33EF-41F7-82E4-B6310A3593CE}" name="Metric Category(s) (Values separated with &quot;;&quot;)" dataDxfId="18"/>
@@ -3143,13 +3134,13 @@
         <v>14</v>
       </c>
       <c r="K1" s="55" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="L1" s="22" t="s">
         <v>15</v>
       </c>
       <c r="M1" s="49" t="s">
-        <v>309</v>
+        <v>330</v>
       </c>
       <c r="N1" s="22" t="s">
         <v>16</v>
@@ -3173,16 +3164,16 @@
         <v>113</v>
       </c>
       <c r="U1" s="59" t="s">
+        <v>324</v>
+      </c>
+      <c r="V1" s="59" t="s">
         <v>325</v>
       </c>
-      <c r="V1" s="59" t="s">
+      <c r="W1" s="59" t="s">
         <v>326</v>
       </c>
-      <c r="W1" s="59" t="s">
+      <c r="X1" s="59" t="s">
         <v>327</v>
-      </c>
-      <c r="X1" s="59" t="s">
-        <v>328</v>
       </c>
       <c r="Y1" s="22" t="s">
         <v>6</v>
@@ -3305,17 +3296,17 @@
       </c>
     </row>
     <row r="3" spans="1:33" ht="60" x14ac:dyDescent="0.25">
-      <c r="A3" s="60" t="s">
+      <c r="A3" s="17" t="s">
+        <v>328</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>244</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>302</v>
+      </c>
+      <c r="D3" s="4" t="s">
         <v>329</v>
-      </c>
-      <c r="B3" s="61" t="s">
-        <v>244</v>
-      </c>
-      <c r="C3" s="61" t="s">
-        <v>302</v>
-      </c>
-      <c r="D3" s="62" t="s">
-        <v>330</v>
       </c>
       <c r="E3" s="15">
         <v>14513.1</v>
@@ -4117,7 +4108,7 @@
         <v>82</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="E12" s="39">
         <v>0.81299999999999994</v>
@@ -4209,7 +4200,7 @@
         <v>91</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="E13" s="38">
         <v>13.41</v>
@@ -4301,7 +4292,7 @@
         <v>96</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="E14" s="40">
         <v>0.96099999999999997</v>
@@ -4389,7 +4380,7 @@
         <v>104</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="E15" s="40">
         <v>3.1E-2</v>
@@ -4477,7 +4468,7 @@
         <v>109</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="E16" s="36">
         <v>0.70199999999999996</v>
@@ -4581,7 +4572,7 @@
         <v>116</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="E17" s="40">
         <v>0.91500000000000004</v>
@@ -4677,7 +4668,7 @@
         <v>121</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="E18" s="40">
         <v>0.69799999999999995</v>
@@ -4757,17 +4748,17 @@
       </c>
     </row>
     <row r="19" spans="1:33" ht="90" x14ac:dyDescent="0.25">
-      <c r="A19" s="60" t="s">
+      <c r="A19" s="17" t="s">
         <v>301</v>
       </c>
-      <c r="B19" s="61" t="s">
+      <c r="B19" s="3" t="s">
         <v>300</v>
       </c>
-      <c r="C19" s="61" t="s">
+      <c r="C19" s="3" t="s">
         <v>264</v>
       </c>
-      <c r="D19" s="62" t="s">
-        <v>312</v>
+      <c r="D19" s="4" t="s">
+        <v>311</v>
       </c>
       <c r="E19" s="36">
         <v>0.68100000000000005</v>
@@ -5136,7 +5127,7 @@
     </row>
     <row r="23" spans="1:33" ht="120" x14ac:dyDescent="0.25">
       <c r="A23" s="18" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="B23" s="5" t="s">
         <v>244</v>
@@ -5145,7 +5136,7 @@
         <v>151</v>
       </c>
       <c r="D23" s="44" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="E23" s="42"/>
       <c r="F23" s="42"/>
@@ -5220,7 +5211,7 @@
     </row>
     <row r="24" spans="1:33" ht="120" x14ac:dyDescent="0.25">
       <c r="A24" s="18" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="B24" s="5" t="s">
         <v>244</v>
@@ -5229,7 +5220,7 @@
         <v>151</v>
       </c>
       <c r="D24" s="44" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="E24" s="42">
         <v>593</v>
@@ -5871,7 +5862,7 @@
         <v>174</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="E31" s="43">
         <v>84.2</v>
@@ -5968,10 +5959,10 @@
         <v>244</v>
       </c>
       <c r="C32" s="4" t="s">
+        <v>321</v>
+      </c>
+      <c r="D32" s="4" t="s">
         <v>322</v>
-      </c>
-      <c r="D32" s="4" t="s">
-        <v>323</v>
       </c>
       <c r="E32" s="43">
         <v>83.6</v>
@@ -6067,7 +6058,7 @@
         <v>185</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="E33" s="43">
         <v>86.4</v>
@@ -6251,7 +6242,7 @@
         <v>303</v>
       </c>
       <c r="D35" s="44" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="E35" s="42">
         <v>2218</v>
@@ -6345,7 +6336,7 @@
         <v>194</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="E36" s="26">
         <v>2648</v>
@@ -6443,7 +6434,7 @@
         <v>201</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="E37" s="26">
         <v>2581</v>
@@ -7047,7 +7038,7 @@
         <v>EMP Baseline (2025-2026 Yr 0)</v>
       </c>
       <c r="M3" s="11" t="str">
-        <v>EMP Target Goal (By YYYY)</v>
+        <v>EMP Target Goal (By 2030)</v>
       </c>
       <c r="N3" s="11" t="str">
         <v>Strategic Plan Baseline (2024-2025 Yr 0)</v>

</xml_diff>